<commit_message>
Add Yahoo lineup records audit workbook data
</commit_message>
<xml_diff>
--- a/Yahoo Starting Lineup Records Audit.xlsx
+++ b/Yahoo Starting Lineup Records Audit.xlsx
@@ -2,8 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Records" sheetId="1" r:id="R8e463de965884f67"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Collection log" sheetId="2" r:id="R652e9cfa2bee4bd4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Records" sheetId="1" r:id="R11ea920dd25348ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Collection log" sheetId="2" r:id="R0a892cbbdf464519"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly candidates" sheetId="3" r:id="Rc7a69dac65f64df4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -123,7 +124,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="28">
+  <x:cellXfs count="30">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -184,6 +185,8 @@
     </x:xf>
     <x:xf numFmtId="201" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -3559,13 +3562,23 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C185" s="27" t="str">
-        <x:v>Not collected</x:v>
-      </x:c>
-      <x:c r="D185" s="26"/>
-      <x:c r="E185" s="27" t="str"/>
-      <x:c r="F185" s="27" t="str"/>
-      <x:c r="G185" s="27" t="str"/>
-      <x:c r="H185" s="27" t="str"/>
+        <x:v>Collected</x:v>
+      </x:c>
+      <x:c r="D185" s="26" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E185" s="27" t="str">
+        <x:v>Dak Prescott — 39.80</x:v>
+      </x:c>
+      <x:c r="F185" s="27" t="str">
+        <x:v>Aaron Jones Sr. — 41.60</x:v>
+      </x:c>
+      <x:c r="G185" s="27" t="str">
+        <x:v>Calvin Ridley — 22.90</x:v>
+      </x:c>
+      <x:c r="H185" s="27" t="str">
+        <x:v>Darren Waller — 16.50</x:v>
+      </x:c>
     </x:row>
     <x:row r="186">
       <x:c r="A186" s="26" t="n">
@@ -4866,4 +4879,597 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="11" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="12" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="12" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="12" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="24" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="12" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="14" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="25" t="str">
+        <x:v>Season</x:v>
+      </x:c>
+      <x:c r="B1" s="25" t="str">
+        <x:v>Week</x:v>
+      </x:c>
+      <x:c r="C1" s="25" t="str">
+        <x:v>Position</x:v>
+      </x:c>
+      <x:c r="D1" s="25" t="str">
+        <x:v>Weekly rank</x:v>
+      </x:c>
+      <x:c r="E1" s="25" t="str">
+        <x:v>Player</x:v>
+      </x:c>
+      <x:c r="F1" s="25" t="str">
+        <x:v>Points</x:v>
+      </x:c>
+      <x:c r="G1" s="25" t="str">
+        <x:v>Lineup slot</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="26" t="n">
+        <x:v>2020</x:v>
+      </x:c>
+      <x:c r="B2" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C2" s="26" t="str">
+        <x:v>QB</x:v>
+      </x:c>
+      <x:c r="D2" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E2" s="27" t="str">
+        <x:v>Russell Wilson</x:v>
+      </x:c>
+      <x:c r="F2" s="29" t="n">
+        <x:v>31.78</x:v>
+      </x:c>
+      <x:c r="G2" s="27" t="str">
+        <x:v>QB</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="26" t="n">
+        <x:v>2020</x:v>
+      </x:c>
+      <x:c r="B3" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C3" s="26" t="str">
+        <x:v>QB</x:v>
+      </x:c>
+      <x:c r="D3" s="26" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E3" s="27" t="str">
+        <x:v>Lamar Jackson</x:v>
+      </x:c>
+      <x:c r="F3" s="29" t="n">
+        <x:v>27.5</x:v>
+      </x:c>
+      <x:c r="G3" s="27" t="str">
+        <x:v>QB</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="26" t="n">
+        <x:v>2020</x:v>
+      </x:c>
+      <x:c r="B4" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C4" s="26" t="str">
+        <x:v>QB</x:v>
+      </x:c>
+      <x:c r="D4" s="26" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E4" s="27" t="str">
+        <x:v>Kyler Murray</x:v>
+      </x:c>
+      <x:c r="F4" s="29" t="n">
+        <x:v>26.3</x:v>
+      </x:c>
+      <x:c r="G4" s="27" t="str">
+        <x:v>QB</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="26" t="n">
+        <x:v>2020</x:v>
+      </x:c>
+      <x:c r="B5" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C5" s="26" t="str">
+        <x:v>RB</x:v>
+      </x:c>
+      <x:c r="D5" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E5" s="27" t="str">
+        <x:v>Josh Jacobs</x:v>
+      </x:c>
+      <x:c r="F5" s="29" t="n">
+        <x:v>31.9</x:v>
+      </x:c>
+      <x:c r="G5" s="27" t="str">
+        <x:v>RB</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="26" t="n">
+        <x:v>2020</x:v>
+      </x:c>
+      <x:c r="B6" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C6" s="26" t="str">
+        <x:v>RB</x:v>
+      </x:c>
+      <x:c r="D6" s="26" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E6" s="27" t="str">
+        <x:v>Christian McCaffrey</x:v>
+      </x:c>
+      <x:c r="F6" s="29" t="n">
+        <x:v>25.5</x:v>
+      </x:c>
+      <x:c r="G6" s="27" t="str">
+        <x:v>RB</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="26" t="n">
+        <x:v>2020</x:v>
+      </x:c>
+      <x:c r="B7" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C7" s="26" t="str">
+        <x:v>RB</x:v>
+      </x:c>
+      <x:c r="D7" s="26" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E7" s="27" t="str">
+        <x:v>Ezekiel Elliott</x:v>
+      </x:c>
+      <x:c r="F7" s="29" t="n">
+        <x:v>24.7</x:v>
+      </x:c>
+      <x:c r="G7" s="27" t="str">
+        <x:v>RB</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="26" t="n">
+        <x:v>2020</x:v>
+      </x:c>
+      <x:c r="B8" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C8" s="26" t="str">
+        <x:v>WR</x:v>
+      </x:c>
+      <x:c r="D8" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E8" s="27" t="str">
+        <x:v>Davante Adams</x:v>
+      </x:c>
+      <x:c r="F8" s="29" t="n">
+        <x:v>27.6</x:v>
+      </x:c>
+      <x:c r="G8" s="27" t="str">
+        <x:v>WR</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="26" t="n">
+        <x:v>2020</x:v>
+      </x:c>
+      <x:c r="B9" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C9" s="26" t="str">
+        <x:v>WR</x:v>
+      </x:c>
+      <x:c r="D9" s="26" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E9" s="27" t="str">
+        <x:v>Adam Thielen</x:v>
+      </x:c>
+      <x:c r="F9" s="29" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="G9" s="27" t="str">
+        <x:v>WR</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="26" t="n">
+        <x:v>2020</x:v>
+      </x:c>
+      <x:c r="B10" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C10" s="26" t="str">
+        <x:v>WR</x:v>
+      </x:c>
+      <x:c r="D10" s="26" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E10" s="27" t="str">
+        <x:v>Calvin Ridley</x:v>
+      </x:c>
+      <x:c r="F10" s="29" t="n">
+        <x:v>24.9</x:v>
+      </x:c>
+      <x:c r="G10" s="27" t="str">
+        <x:v>WR</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="26" t="n">
+        <x:v>2020</x:v>
+      </x:c>
+      <x:c r="B11" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C11" s="26" t="str">
+        <x:v>TE</x:v>
+      </x:c>
+      <x:c r="D11" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E11" s="27" t="str">
+        <x:v>Mark Andrews</x:v>
+      </x:c>
+      <x:c r="F11" s="29" t="n">
+        <x:v>17.8</x:v>
+      </x:c>
+      <x:c r="G11" s="27" t="str">
+        <x:v>TE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="26" t="n">
+        <x:v>2020</x:v>
+      </x:c>
+      <x:c r="B12" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C12" s="26" t="str">
+        <x:v>TE</x:v>
+      </x:c>
+      <x:c r="D12" s="26" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E12" s="27" t="str">
+        <x:v>T.J. Hockenson</x:v>
+      </x:c>
+      <x:c r="F12" s="29" t="n">
+        <x:v>11.6</x:v>
+      </x:c>
+      <x:c r="G12" s="27" t="str">
+        <x:v>TE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="26" t="n">
+        <x:v>2020</x:v>
+      </x:c>
+      <x:c r="B13" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C13" s="26" t="str">
+        <x:v>TE</x:v>
+      </x:c>
+      <x:c r="D13" s="26" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E13" s="27" t="str">
+        <x:v>Travis Kelce</x:v>
+      </x:c>
+      <x:c r="F13" s="29" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="G13" s="27" t="str">
+        <x:v>TE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="26" t="n">
+        <x:v>2020</x:v>
+      </x:c>
+      <x:c r="B14" s="26" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C14" s="26" t="str">
+        <x:v>QB</x:v>
+      </x:c>
+      <x:c r="D14" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E14" s="27" t="str">
+        <x:v>Dak Prescott</x:v>
+      </x:c>
+      <x:c r="F14" s="29" t="n">
+        <x:v>39.8</x:v>
+      </x:c>
+      <x:c r="G14" s="27" t="str">
+        <x:v>QB</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="26" t="n">
+        <x:v>2020</x:v>
+      </x:c>
+      <x:c r="B15" s="26" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C15" s="26" t="str">
+        <x:v>QB</x:v>
+      </x:c>
+      <x:c r="D15" s="26" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E15" s="27" t="str">
+        <x:v>Cam Newton</x:v>
+      </x:c>
+      <x:c r="F15" s="29" t="n">
+        <x:v>34.58</x:v>
+      </x:c>
+      <x:c r="G15" s="27" t="str">
+        <x:v>QB</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="26" t="n">
+        <x:v>2020</x:v>
+      </x:c>
+      <x:c r="B16" s="26" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C16" s="26" t="str">
+        <x:v>QB</x:v>
+      </x:c>
+      <x:c r="D16" s="26" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E16" s="27" t="str">
+        <x:v>Josh Allen</x:v>
+      </x:c>
+      <x:c r="F16" s="29" t="n">
+        <x:v>34.5</x:v>
+      </x:c>
+      <x:c r="G16" s="27" t="str">
+        <x:v>QB</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="26" t="n">
+        <x:v>2020</x:v>
+      </x:c>
+      <x:c r="B17" s="26" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C17" s="26" t="str">
+        <x:v>RB</x:v>
+      </x:c>
+      <x:c r="D17" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E17" s="27" t="str">
+        <x:v>Aaron Jones Sr.</x:v>
+      </x:c>
+      <x:c r="F17" s="29" t="n">
+        <x:v>41.6</x:v>
+      </x:c>
+      <x:c r="G17" s="27" t="str">
+        <x:v>W/R/T</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="26" t="n">
+        <x:v>2020</x:v>
+      </x:c>
+      <x:c r="B18" s="26" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C18" s="26" t="str">
+        <x:v>RB</x:v>
+      </x:c>
+      <x:c r="D18" s="26" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E18" s="27" t="str">
+        <x:v>Alvin Kamara</x:v>
+      </x:c>
+      <x:c r="F18" s="29" t="n">
+        <x:v>29.4</x:v>
+      </x:c>
+      <x:c r="G18" s="27" t="str">
+        <x:v>RB</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="26" t="n">
+        <x:v>2020</x:v>
+      </x:c>
+      <x:c r="B19" s="26" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C19" s="26" t="str">
+        <x:v>RB</x:v>
+      </x:c>
+      <x:c r="D19" s="26" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E19" s="27" t="str">
+        <x:v>Nick Chubb</x:v>
+      </x:c>
+      <x:c r="F19" s="29" t="n">
+        <x:v>25.3</x:v>
+      </x:c>
+      <x:c r="G19" s="27" t="str">
+        <x:v>RB</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="26" t="n">
+        <x:v>2020</x:v>
+      </x:c>
+      <x:c r="B20" s="26" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C20" s="26" t="str">
+        <x:v>WR</x:v>
+      </x:c>
+      <x:c r="D20" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E20" s="27" t="str">
+        <x:v>Calvin Ridley</x:v>
+      </x:c>
+      <x:c r="F20" s="29" t="n">
+        <x:v>22.9</x:v>
+      </x:c>
+      <x:c r="G20" s="27" t="str">
+        <x:v>WR</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="26" t="n">
+        <x:v>2020</x:v>
+      </x:c>
+      <x:c r="B21" s="26" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C21" s="26" t="str">
+        <x:v>WR</x:v>
+      </x:c>
+      <x:c r="D21" s="26" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E21" s="27" t="str">
+        <x:v>Stefon Diggs</x:v>
+      </x:c>
+      <x:c r="F21" s="29" t="n">
+        <x:v>21.3</x:v>
+      </x:c>
+      <x:c r="G21" s="27" t="str">
+        <x:v>WR</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="26" t="n">
+        <x:v>2020</x:v>
+      </x:c>
+      <x:c r="B22" s="26" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C22" s="26" t="str">
+        <x:v>WR</x:v>
+      </x:c>
+      <x:c r="D22" s="26" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E22" s="27" t="str">
+        <x:v>Terry McLaurin</x:v>
+      </x:c>
+      <x:c r="F22" s="29" t="n">
+        <x:v>18.5</x:v>
+      </x:c>
+      <x:c r="G22" s="27" t="str">
+        <x:v>WR</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="26" t="n">
+        <x:v>2020</x:v>
+      </x:c>
+      <x:c r="B23" s="26" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C23" s="26" t="str">
+        <x:v>TE</x:v>
+      </x:c>
+      <x:c r="D23" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E23" s="27" t="str">
+        <x:v>Darren Waller</x:v>
+      </x:c>
+      <x:c r="F23" s="29" t="n">
+        <x:v>16.5</x:v>
+      </x:c>
+      <x:c r="G23" s="27" t="str">
+        <x:v>TE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="26" t="n">
+        <x:v>2020</x:v>
+      </x:c>
+      <x:c r="B24" s="26" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C24" s="26" t="str">
+        <x:v>TE</x:v>
+      </x:c>
+      <x:c r="D24" s="26" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E24" s="27" t="str">
+        <x:v>Travis Kelce</x:v>
+      </x:c>
+      <x:c r="F24" s="29" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="G24" s="27" t="str">
+        <x:v>TE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="26" t="n">
+        <x:v>2020</x:v>
+      </x:c>
+      <x:c r="B25" s="26" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C25" s="26" t="str">
+        <x:v>TE</x:v>
+      </x:c>
+      <x:c r="D25" s="26" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E25" s="27" t="str">
+        <x:v>Noah Fant</x:v>
+      </x:c>
+      <x:c r="F25" s="29" t="n">
+        <x:v>13.7</x:v>
+      </x:c>
+      <x:c r="G25" s="27" t="str">
+        <x:v>TE</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>

<commit_message>
Update Yahoo lineup audit workbook and collection log
</commit_message>
<xml_diff>
--- a/Yahoo Starting Lineup Records Audit.xlsx
+++ b/Yahoo Starting Lineup Records Audit.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Records" sheetId="1" r:id="R11ea920dd25348ae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Collection log" sheetId="2" r:id="R0a892cbbdf464519"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly candidates" sheetId="3" r:id="Rc7a69dac65f64df4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Records" sheetId="1" r:id="R3b6252186ba04c56"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Collection log" sheetId="2" r:id="Rcf73992953994b96"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly candidates" sheetId="3" r:id="Rdf9a6dc9d31c4c50"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3588,13 +3588,23 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C186" s="27" t="str">
-        <x:v>Not collected</x:v>
-      </x:c>
-      <x:c r="D186" s="26"/>
-      <x:c r="E186" s="27" t="str"/>
-      <x:c r="F186" s="27" t="str"/>
-      <x:c r="G186" s="27" t="str"/>
-      <x:c r="H186" s="27" t="str"/>
+        <x:v>Collected</x:v>
+      </x:c>
+      <x:c r="D186" s="26" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E186" s="27" t="str">
+        <x:v>Patrick Mahomes — 40.00</x:v>
+      </x:c>
+      <x:c r="F186" s="27" t="str">
+        <x:v>Alvin Kamara — 31.70</x:v>
+      </x:c>
+      <x:c r="G186" s="27" t="str">
+        <x:v>Tyler Lockett — 28.00</x:v>
+      </x:c>
+      <x:c r="H186" s="27" t="str">
+        <x:v>Travis Kelce — 8.70</x:v>
+      </x:c>
     </x:row>
     <x:row r="187">
       <x:c r="A187" s="26" t="n">
@@ -5469,6 +5479,282 @@
         <x:v>TE</x:v>
       </x:c>
     </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="26" t="n">
+        <x:v>2020</x:v>
+      </x:c>
+      <x:c r="B26" s="26" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C26" s="26" t="str">
+        <x:v>QB</x:v>
+      </x:c>
+      <x:c r="D26" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E26" s="27" t="str">
+        <x:v>Patrick Mahomes</x:v>
+      </x:c>
+      <x:c r="F26" s="29" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="G26" s="27" t="str">
+        <x:v>QB</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="26" t="n">
+        <x:v>2020</x:v>
+      </x:c>
+      <x:c r="B27" s="26" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C27" s="26" t="str">
+        <x:v>QB</x:v>
+      </x:c>
+      <x:c r="D27" s="26" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E27" s="27" t="str">
+        <x:v>Russell Wilson</x:v>
+      </x:c>
+      <x:c r="F27" s="29" t="n">
+        <x:v>36.8</x:v>
+      </x:c>
+      <x:c r="G27" s="27" t="str">
+        <x:v>QB</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="26" t="n">
+        <x:v>2020</x:v>
+      </x:c>
+      <x:c r="B28" s="26" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C28" s="26" t="str">
+        <x:v>QB</x:v>
+      </x:c>
+      <x:c r="D28" s="26" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E28" s="27" t="str">
+        <x:v>Josh Allen</x:v>
+      </x:c>
+      <x:c r="F28" s="29" t="n">
+        <x:v>31.24</x:v>
+      </x:c>
+      <x:c r="G28" s="27" t="str">
+        <x:v>QB</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="26" t="n">
+        <x:v>2020</x:v>
+      </x:c>
+      <x:c r="B29" s="26" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C29" s="26" t="str">
+        <x:v>RB</x:v>
+      </x:c>
+      <x:c r="D29" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E29" s="27" t="str">
+        <x:v>Alvin Kamara</x:v>
+      </x:c>
+      <x:c r="F29" s="29" t="n">
+        <x:v>31.7</x:v>
+      </x:c>
+      <x:c r="G29" s="27" t="str">
+        <x:v>RB</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="26" t="n">
+        <x:v>2020</x:v>
+      </x:c>
+      <x:c r="B30" s="26" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C30" s="26" t="str">
+        <x:v>RB</x:v>
+      </x:c>
+      <x:c r="D30" s="26" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E30" s="27" t="str">
+        <x:v>Derrick Henry</x:v>
+      </x:c>
+      <x:c r="F30" s="29" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="G30" s="27" t="str">
+        <x:v>RB</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="26" t="n">
+        <x:v>2020</x:v>
+      </x:c>
+      <x:c r="B31" s="26" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C31" s="26" t="str">
+        <x:v>RB</x:v>
+      </x:c>
+      <x:c r="D31" s="26" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E31" s="27" t="str">
+        <x:v>Dalvin Cook</x:v>
+      </x:c>
+      <x:c r="F31" s="29" t="n">
+        <x:v>23.9</x:v>
+      </x:c>
+      <x:c r="G31" s="27" t="str">
+        <x:v>RB</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="26" t="n">
+        <x:v>2020</x:v>
+      </x:c>
+      <x:c r="B32" s="26" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C32" s="26" t="str">
+        <x:v>WR</x:v>
+      </x:c>
+      <x:c r="D32" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E32" s="27" t="str">
+        <x:v>Tyler Lockett</x:v>
+      </x:c>
+      <x:c r="F32" s="29" t="n">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="G32" s="27" t="str">
+        <x:v>WR</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="26" t="n">
+        <x:v>2020</x:v>
+      </x:c>
+      <x:c r="B33" s="26" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C33" s="26" t="str">
+        <x:v>WR</x:v>
+      </x:c>
+      <x:c r="D33" s="26" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E33" s="27" t="str">
+        <x:v>Michael Gallup</x:v>
+      </x:c>
+      <x:c r="F33" s="29" t="n">
+        <x:v>19.8</x:v>
+      </x:c>
+      <x:c r="G33" s="27" t="str">
+        <x:v>WR</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="26" t="n">
+        <x:v>2020</x:v>
+      </x:c>
+      <x:c r="B34" s="26" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C34" s="26" t="str">
+        <x:v>WR</x:v>
+      </x:c>
+      <x:c r="D34" s="26" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E34" s="27" t="str">
+        <x:v>Keenan Allen</x:v>
+      </x:c>
+      <x:c r="F34" s="29" t="n">
+        <x:v>17.2</x:v>
+      </x:c>
+      <x:c r="G34" s="27" t="str">
+        <x:v>WR</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="26" t="n">
+        <x:v>2020</x:v>
+      </x:c>
+      <x:c r="B35" s="26" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C35" s="26" t="str">
+        <x:v>TE</x:v>
+      </x:c>
+      <x:c r="D35" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E35" s="27" t="str">
+        <x:v>Travis Kelce</x:v>
+      </x:c>
+      <x:c r="F35" s="29" t="n">
+        <x:v>8.7</x:v>
+      </x:c>
+      <x:c r="G35" s="27" t="str">
+        <x:v>TE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="26" t="n">
+        <x:v>2020</x:v>
+      </x:c>
+      <x:c r="B36" s="26" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C36" s="26" t="str">
+        <x:v>TE</x:v>
+      </x:c>
+      <x:c r="D36" s="26" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E36" s="27" t="str">
+        <x:v>Mike Gesicki</x:v>
+      </x:c>
+      <x:c r="F36" s="29" t="n">
+        <x:v>7.5</x:v>
+      </x:c>
+      <x:c r="G36" s="27" t="str">
+        <x:v>TE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="26" t="n">
+        <x:v>2020</x:v>
+      </x:c>
+      <x:c r="B37" s="26" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C37" s="26" t="str">
+        <x:v>TE</x:v>
+      </x:c>
+      <x:c r="D37" s="26" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E37" s="27" t="str">
+        <x:v>Zach Ertz</x:v>
+      </x:c>
+      <x:c r="F37" s="29" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="G37" s="27" t="str">
+        <x:v>TE</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>